<commit_message>
reply comment nriss 80f07324fa8f25986cd42ed6e59a506f7b70e1f3
</commit_message>
<xml_diff>
--- a/cp-ins-iti-105/ig/StructureDefinition-pdsm-simplified-publish.xlsx
+++ b/cp-ins-iti-105/ig/StructureDefinition-pdsm-simplified-publish.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="525">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T08:31:43+00:00</t>
+    <t>2026-07-30T10:07:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1625,6 +1625,10 @@
   </si>
   <si>
     <t>DocumentReference.context.sourcePatientInfo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient) &lt;&lt;contained&gt;&gt;
+</t>
   </si>
   <si>
     <t>Référence vers la ressource Patient titulaire du dossier. Conformément à IHE MHD ITI-105, lorsque fournie, cette référence pointe une ressource Patient contenue (contained). Selon le statut d'identité, la ressource est conforme au profil FR Core Patient (identité non qualifiée) ou FR Core Patient INS (identité qualifiée, matricule INS + traits INSi) qui hérite de profil FR Core Patient.</t>
@@ -9671,13 +9675,13 @@
         <v>80</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>267</v>
+        <v>511</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -9740,7 +9744,7 @@
         <v>80</v>
       </c>
       <c r="AJ63" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="AK63" t="s" s="2">
         <v>80</v>
@@ -9761,15 +9765,15 @@
         <v>80</v>
       </c>
       <c r="AQ63" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9792,16 +9796,16 @@
         <v>80</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="N64" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
@@ -9851,7 +9855,7 @@
         <v>80</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>81</v>
@@ -9869,13 +9873,13 @@
         <v>80</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="AM64" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AO64" t="s" s="2">
         <v>80</v>
@@ -9884,7 +9888,7 @@
         <v>80</v>
       </c>
       <c r="AQ64" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
   </sheetData>

</xml_diff>